<commit_message>
Office 模板换成新墨色 #38352F（OneHistory 统一配色 2026-10-23）
</commit_message>
<xml_diff>
--- a/z-Unused/b-Office/BOM表.xlsx
+++ b/z-Unused/b-Office/BOM表.xlsx
@@ -186,7 +186,7 @@
     <font>
       <b/>
       <sz val="16"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
@@ -194,33 +194,33 @@
     <font>
       <b/>
       <sz val="9.5"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Bahnschrift"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF6A6458"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF6A6458"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
@@ -228,26 +228,26 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Bahnschrift"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF6A6458"/>
+      <color rgb="FF38352F"/>
       <name val="Bahnschrift"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF26231E"/>
+      <color rgb="FF38352F"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
@@ -286,10 +286,10 @@
       <left/>
       <right/>
       <top style="thick">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -299,10 +299,10 @@
       </left>
       <right/>
       <top style="thick">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -331,7 +331,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -342,7 +342,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -350,7 +350,7 @@
       <left/>
       <right/>
       <top style="thick">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -361,7 +361,7 @@
       </left>
       <right/>
       <top style="thick">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -371,7 +371,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -382,7 +382,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -390,7 +390,7 @@
       <left/>
       <right/>
       <top style="thick">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -401,7 +401,7 @@
       </left>
       <right/>
       <top style="thick">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -411,7 +411,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -422,7 +422,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -435,7 +435,7 @@
         <color rgb="FFD5D1C8"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -443,10 +443,10 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -454,10 +454,10 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF26231E"/>
+        <color rgb="FF38352F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -634,7 +634,7 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="26231E"/>
+          <a:srgbClr val="38352F"/>
         </a:solidFill>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:noFill/>
@@ -754,7 +754,7 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="26231E"/>
+          <a:srgbClr val="38352F"/>
         </a:solidFill>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:noFill/>

</xml_diff>